<commit_message>
Mark 1808 as sold for 500
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -134,8 +134,18 @@
       <family val="2"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <strike val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -232,8 +242,26 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCC0DA"/>
+        <bgColor rgb="00CCC0DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -301,11 +329,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -413,6 +455,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2545,25 +2599,25 @@
       <c r="E83" s="25" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B84" s="23" t="inlineStr">
+      <c r="A84" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B84" s="38" t="inlineStr">
         <is>
           <t>#1808</t>
         </is>
       </c>
-      <c r="C84" s="23" t="inlineStr">
+      <c r="C84" s="38" t="inlineStr">
         <is>
           <t>Mr. Whatsit (Season 5)</t>
         </is>
       </c>
-      <c r="D84" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E84" s="25" t="n"/>
+      <c r="D84" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E84" s="39" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="23" t="inlineStr">
@@ -2681,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -2915,6 +2969,21 @@
         <v>2100</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>#1808 Mr. Whatsit (Season 5)</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="n">
+        <v>500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 1462 (Sticker), 1778, 1797 as sold for 1800
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -2011,25 +2011,25 @@
       <c r="E55" s="25" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B56" s="18" t="inlineStr">
+      <c r="A56" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B56" s="38" t="inlineStr">
         <is>
           <t>#1462</t>
         </is>
       </c>
-      <c r="C56" s="18" t="inlineStr">
+      <c r="C56" s="38" t="inlineStr">
         <is>
           <t>Eddie (Special Edition 顛倒世界戰鬥 - 有貼紙)</t>
         </is>
       </c>
-      <c r="D56" s="18" t="n">
+      <c r="D56" s="38" t="n">
         <v>800</v>
       </c>
-      <c r="E56" s="19" t="n"/>
+      <c r="E56" s="39" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
@@ -2305,25 +2305,25 @@
       <c r="E69" s="22" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B70" s="18" t="inlineStr">
+      <c r="A70" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B70" s="38" t="inlineStr">
         <is>
           <t>#1778</t>
         </is>
       </c>
-      <c r="C70" s="18" t="inlineStr">
+      <c r="C70" s="38" t="inlineStr">
         <is>
           <t>Nancy Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D70" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E70" s="19" t="n"/>
+      <c r="D70" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E70" s="39" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="23" t="inlineStr">
@@ -2494,25 +2494,25 @@
       <c r="E78" s="19" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B79" s="18" t="inlineStr">
+      <c r="A79" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B79" s="38" t="inlineStr">
         <is>
           <t>#1797</t>
         </is>
       </c>
-      <c r="C79" s="18" t="inlineStr">
+      <c r="C79" s="38" t="inlineStr">
         <is>
           <t>Jonathan Byers (Season 5)</t>
         </is>
       </c>
-      <c r="D79" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E79" s="19" t="n"/>
+      <c r="D79" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E79" s="39" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="23" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -2984,6 +2984,23 @@
         <v>500</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>#1462 Eddie (Special Edition 顛倒世界戰鬥 - 有貼紙)
+#1778 Nancy Wheeler (Season 5)
+#1797 Jonathan Byers (Season 5)</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="n">
+        <v>1800</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 804 as sold on 2026-09-03 for 650 in Excel
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -1568,25 +1568,25 @@
       <c r="E34" s="25" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
         <is>
           <t>#804</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C35" s="38" t="inlineStr">
         <is>
           <t>Dustin (Walmart 限定 夏令營帽子)</t>
         </is>
       </c>
-      <c r="D35" s="24" t="n">
+      <c r="D35" s="38" t="n">
         <v>650</v>
       </c>
-      <c r="E35" s="25" t="n"/>
+      <c r="E35" s="39" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3001,6 +3001,21 @@
         <v>1800</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>#804 Dustin (Walmart 限定 夏令營帽子)</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="n">
+        <v>650</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 7 items as sold for 3600
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -1188,25 +1188,25 @@
       <c r="E16" s="25" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>#514</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="38" t="inlineStr">
         <is>
           <t>Nancy (第一季拿槍款)</t>
         </is>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="38" t="n">
         <v>750</v>
       </c>
-      <c r="E17" s="25" t="n"/>
+      <c r="E17" s="39" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
@@ -1358,46 +1358,46 @@
       <c r="E24" s="19" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
         <is>
           <t>#640</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="38" t="inlineStr">
         <is>
           <t>Billy (比利經典款)</t>
         </is>
       </c>
-      <c r="D25" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E25" s="25" t="n"/>
+      <c r="D25" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E25" s="39" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>#643</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="38" t="inlineStr">
         <is>
           <t>Vampire Bob (吸血鬼鮑伯)</t>
         </is>
       </c>
-      <c r="D26" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E26" s="25" t="n"/>
+      <c r="D26" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E26" s="39" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
@@ -1759,25 +1759,25 @@
       <c r="E43" s="25" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="20" t="inlineStr">
+      <c r="A44" s="38" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B44" s="38" t="inlineStr">
         <is>
           <t>Deluxe #1186</t>
         </is>
       </c>
-      <c r="C44" s="20" t="inlineStr">
+      <c r="C44" s="38" t="inlineStr">
         <is>
           <t>Byers House: Demogorgon (拜爾斯家魔王破牆)</t>
         </is>
       </c>
-      <c r="D44" s="21" t="n">
+      <c r="D44" s="38" t="n">
         <v>1000</v>
       </c>
-      <c r="E44" s="22" t="n"/>
+      <c r="E44" s="39" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="28" t="inlineStr">
@@ -1843,25 +1843,25 @@
       <c r="E47" s="17" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="15" t="inlineStr">
+      <c r="A48" s="38" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B48" s="38" t="inlineStr">
         <is>
           <t>#1250</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="C48" s="38" t="inlineStr">
         <is>
           <t>Eddie (Target 限定 經典吉他版)</t>
         </is>
       </c>
-      <c r="D48" s="16" t="n">
+      <c r="D48" s="38" t="n">
         <v>800</v>
       </c>
-      <c r="E48" s="17" t="n"/>
+      <c r="E48" s="39" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
@@ -1885,25 +1885,25 @@
       <c r="E49" s="19" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B50" s="23" t="inlineStr">
+      <c r="A50" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B50" s="38" t="inlineStr">
         <is>
           <t>#1301</t>
         </is>
       </c>
-      <c r="C50" s="23" t="inlineStr">
+      <c r="C50" s="38" t="inlineStr">
         <is>
           <t>Erica (S4 戰鬥裝備)</t>
         </is>
       </c>
-      <c r="D50" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E50" s="25" t="n"/>
+      <c r="D50" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E50" s="39" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
@@ -2368,25 +2368,25 @@
       <c r="E72" s="25" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B73" s="23" t="inlineStr">
+      <c r="A73" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B73" s="38" t="inlineStr">
         <is>
           <t>#1782</t>
         </is>
       </c>
-      <c r="C73" s="23" t="inlineStr">
+      <c r="C73" s="38" t="inlineStr">
         <is>
           <t>Holly Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D73" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E73" s="25" t="n"/>
+      <c r="D73" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E73" s="39" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="23" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3016,6 +3016,27 @@
         <v>650</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>#514 Nancy (第一季拿槍款)
+#640 Billy (比利經典款)
+#643 Vampire Bob (吸血鬼鮑伯)
+Deluxe #1186 Byers House: Demogorgon (拜爾斯家魔王破牆)
+#1250 Eddie (Target 限定 經典吉他版)
+#1301 Erica (S4 戰鬥裝備)
+#1782 Holly Wheeler (Season 5)</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="n">
+        <v>3600</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update 1808 price to 400
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D84" s="38" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="E84" s="39" t="n"/>
     </row>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="C13" s="41" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Mark 1798 and 1802 as sold for 1000
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -2515,46 +2515,46 @@
       <c r="E79" s="39" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B80" s="23" t="inlineStr">
+      <c r="A80" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B80" s="38" t="inlineStr">
         <is>
           <t>#1798</t>
         </is>
       </c>
-      <c r="C80" s="23" t="inlineStr">
+      <c r="C80" s="38" t="inlineStr">
         <is>
           <t>Lucas Sinclair (S5 WSQK 特別款)</t>
         </is>
       </c>
-      <c r="D80" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E80" s="25" t="n"/>
+      <c r="D80" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E80" s="39" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B81" s="23" t="inlineStr">
+      <c r="A81" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B81" s="38" t="inlineStr">
         <is>
           <t>#1802</t>
         </is>
       </c>
-      <c r="C81" s="23" t="inlineStr">
+      <c r="C81" s="38" t="inlineStr">
         <is>
           <t>Nancy Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D81" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E81" s="25" t="n"/>
+      <c r="D81" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E81" s="39" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="23" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3037,6 +3037,22 @@
         <v>3600</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B17" s="41" t="inlineStr">
+        <is>
+          <t>#1798 Lucas Sinclair (S5 WSQK 特別款)
+#1802 Nancy Wheeler (Season 5)</t>
+        </is>
+      </c>
+      <c r="C17" s="41" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 428, 720, 1810 as sold for 1200 (80% off price)
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -1083,25 +1083,25 @@
       <c r="E11" s="25" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>#428</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Demogorgon (魔王開口款)</t>
         </is>
       </c>
-      <c r="D12" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E12" s="25" t="n"/>
+      <c r="D12" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E12" s="39" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
@@ -1463,25 +1463,25 @@
       <c r="E29" s="19" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="inlineStr">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
         <is>
           <t>#720</t>
         </is>
       </c>
-      <c r="C30" s="23" t="inlineStr">
+      <c r="C30" s="38" t="inlineStr">
         <is>
           <t>Hopper (約會襯衫款)</t>
         </is>
       </c>
-      <c r="D30" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E30" s="25" t="n"/>
+      <c r="D30" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E30" s="39" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
@@ -2620,25 +2620,25 @@
       <c r="E84" s="39" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B85" s="23" t="inlineStr">
+      <c r="A85" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B85" s="38" t="inlineStr">
         <is>
           <t>#1810</t>
         </is>
       </c>
-      <c r="C85" s="23" t="inlineStr">
+      <c r="C85" s="38" t="inlineStr">
         <is>
           <t>Holly The Heroic (S5 英雄霍莉)</t>
         </is>
       </c>
-      <c r="D85" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E85" s="25" t="n"/>
+      <c r="D85" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E85" s="39" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="35" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3053,6 +3053,23 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>#428 Demogorgon (魔王開口款)
+#720 Hopper (約會襯衫款)
+#1810 Holly The Heroic (S5 英雄霍莉)</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="n">
+        <v>1200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 10 items as sold for 6500
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -1125,25 +1125,25 @@
       <c r="E13" s="32" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>#476</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
         <is>
           <t>Mr. Clarke (2017 SDCC 展會限定)</t>
         </is>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="38" t="n">
         <v>1500</v>
       </c>
-      <c r="E14" s="17" t="n"/>
+      <c r="E14" s="39" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
@@ -1167,25 +1167,25 @@
       <c r="E15" s="25" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>#513</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="38" t="inlineStr">
         <is>
           <t>Jonathan (第一季照相機)</t>
         </is>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="38" t="n">
         <v>750</v>
       </c>
-      <c r="E16" s="25" t="n"/>
+      <c r="E16" s="39" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
@@ -1209,25 +1209,25 @@
       <c r="E17" s="39" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>#515</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="38" t="inlineStr">
         <is>
           <t>Brenner (布倫納博士)</t>
         </is>
       </c>
-      <c r="D18" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E18" s="25" t="n"/>
+      <c r="D18" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E18" s="39" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
@@ -1272,27 +1272,27 @@
       <c r="E20" s="25" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>#572</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="38" t="inlineStr">
         <is>
           <t>Eleven (BoxLunch 限定 吊帶褲)</t>
         </is>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D21" s="38" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="E21" s="25" t="n"/>
+      <c r="E21" s="39" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
@@ -1316,25 +1316,25 @@
       <c r="E22" s="19" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="A23" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>#637</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="38" t="inlineStr">
         <is>
           <t>Eleven (Elevated 升空施法)</t>
         </is>
       </c>
-      <c r="D23" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E23" s="25" t="n"/>
+      <c r="D23" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E23" s="39" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -2704,25 +2704,25 @@
       <c r="E88" s="17" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="15" t="inlineStr">
+      <c r="A89" s="38" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B89" s="15" t="inlineStr">
+      <c r="B89" s="38" t="inlineStr">
         <is>
           <t>套組</t>
         </is>
       </c>
-      <c r="C89" s="15" t="inlineStr">
+      <c r="C89" s="38" t="inlineStr">
         <is>
           <t>Vecna &amp; Vecna 雙入組 (2022 NYCC 展會限定)</t>
         </is>
       </c>
-      <c r="D89" s="16" t="n">
+      <c r="D89" s="38" t="n">
         <v>900</v>
       </c>
-      <c r="E89" s="17" t="n"/>
+      <c r="E89" s="39" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3070,6 +3070,26 @@
         <v>1200</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>#476 Mr. Clarke (2017 SDCC 展會限定)
+#513 Jonathan (第一季照相機)
+#515 Brenner (布倫納博士)
+#572 Eleven (BoxLunch 限定 吊帶褲)
+#637 Eleven (Elevated 升空施法)
+套組 Vecna &amp; Vecna 雙入組 (2022 NYCC 展會限定)</t>
+        </is>
+      </c>
+      <c r="C19" s="41" t="n">
+        <v>6500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 546-549 bundle as sold in Excel
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -2662,25 +2662,25 @@
       <c r="E86" s="37" t="n"/>
     </row>
     <row r="87" ht="15.3" customHeight="1">
-      <c r="A87" s="15" t="inlineStr">
+      <c r="A87" s="38" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B87" s="15" t="inlineStr">
+      <c r="B87" s="38" t="inlineStr">
         <is>
           <t>套組</t>
         </is>
       </c>
-      <c r="C87" s="15" t="inlineStr">
+      <c r="C87" s="38" t="inlineStr">
         <is>
           <t>捉鬼敢死隊 4 人組 (#546, #547, #548, #549)</t>
         </is>
       </c>
-      <c r="D87" s="16" t="n">
+      <c r="D87" s="38" t="n">
         <v>3700</v>
       </c>
-      <c r="E87" s="17" t="n"/>
+      <c r="E87" s="39" t="n"/>
     </row>
     <row r="88" ht="15.3" customHeight="1">
       <c r="A88" s="15" t="inlineStr">
@@ -3083,7 +3083,8 @@
 #515 Brenner (布倫納博士)
 #572 Eleven (BoxLunch 限定 吊帶褲)
 #637 Eleven (Elevated 升空施法)
-套組 Vecna &amp; Vecna 雙入組 (2022 NYCC 展會限定)</t>
+套組 Vecna &amp; Vecna 雙入組 (2022 NYCC 展會限定)
+套組 捉鬼敢死隊 4 人組 (#546, #547, #548, #549)</t>
         </is>
       </c>
       <c r="C19" s="41" t="n">

</xml_diff>

<commit_message>
Mark 550 as sold for 400
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -1251,25 +1251,25 @@
       <c r="E19" s="25" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>#550</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="38" t="inlineStr">
         <is>
           <t>Joyce (磁鐵版)</t>
         </is>
       </c>
-      <c r="D20" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E20" s="25" t="n"/>
+      <c r="D20" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E20" s="39" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3091,6 +3091,21 @@
         <v>6500</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>#550 Joyce (磁鐵版)</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="n">
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Swap 720 for 512 in sales record and inventory
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -144,8 +144,14 @@
       <name val="微軟正黑體"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <strike val="0"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -260,6 +266,12 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+        <bgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -347,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -467,6 +479,12 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="19" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1146,25 +1164,25 @@
       <c r="E14" s="39" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>#512</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="38" t="inlineStr">
         <is>
           <t>Hopper (警長常規款)</t>
         </is>
       </c>
-      <c r="D15" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E15" s="25" t="n"/>
+      <c r="D15" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E15" s="39" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
@@ -1463,25 +1481,25 @@
       <c r="E29" s="19" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B30" s="38" t="inlineStr">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
         <is>
           <t>#720</t>
         </is>
       </c>
-      <c r="C30" s="38" t="inlineStr">
+      <c r="C30" s="42" t="inlineStr">
         <is>
           <t>Hopper (約會襯衫款)</t>
         </is>
       </c>
-      <c r="D30" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E30" s="39" t="n"/>
+      <c r="D30" s="42" t="n">
+        <v>500</v>
+      </c>
+      <c r="E30" s="43" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
@@ -3062,7 +3080,7 @@
       <c r="B18" s="41" t="inlineStr">
         <is>
           <t>#428 Demogorgon (魔王開口款)
-#720 Hopper (約會襯衫款)
+#512 Hopper (警長常規款)
 #1810 Holly The Heroic (S5 英雄霍莉)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Mark 1780 and 1783 as sold for 800
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -2344,25 +2344,25 @@
       <c r="E70" s="39" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B71" s="23" t="inlineStr">
+      <c r="A71" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B71" s="38" t="inlineStr">
         <is>
           <t>#1780</t>
         </is>
       </c>
-      <c r="C71" s="23" t="inlineStr">
+      <c r="C71" s="38" t="inlineStr">
         <is>
           <t>Eleven (Season 5)</t>
         </is>
       </c>
-      <c r="D71" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E71" s="25" t="n"/>
+      <c r="D71" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E71" s="39" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="23" t="inlineStr">
@@ -2407,25 +2407,25 @@
       <c r="E73" s="39" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B74" s="23" t="inlineStr">
+      <c r="A74" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B74" s="38" t="inlineStr">
         <is>
           <t>#1783</t>
         </is>
       </c>
-      <c r="C74" s="23" t="inlineStr">
+      <c r="C74" s="38" t="inlineStr">
         <is>
           <t>Mike Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D74" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E74" s="25" t="n"/>
+      <c r="D74" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E74" s="39" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="23" t="inlineStr">
@@ -2753,7 +2753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3124,6 +3124,22 @@
         <v>400</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B21" s="41" t="inlineStr">
+        <is>
+          <t>#1780 Eleven (Season 5)
+#1783 Mike Wheeler (Season 5)</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="n">
+        <v>800</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 803 and 922 as sold for 800
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -1565,25 +1565,25 @@
       <c r="E33" s="19" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B34" s="23" t="inlineStr">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>#803</t>
         </is>
       </c>
-      <c r="C34" s="23" t="inlineStr">
+      <c r="C34" s="38" t="inlineStr">
         <is>
           <t>Steve (拿聖代冰淇淋款)</t>
         </is>
       </c>
-      <c r="D34" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E34" s="25" t="n"/>
+      <c r="D34" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E34" s="39" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
@@ -1756,25 +1756,25 @@
       <c r="E42" s="17" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B43" s="23" t="inlineStr">
+      <c r="A43" s="38" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
         <is>
           <t>#922</t>
         </is>
       </c>
-      <c r="C43" s="23" t="inlineStr">
+      <c r="C43" s="38" t="inlineStr">
         <is>
           <t>Robin (拿白板款)</t>
         </is>
       </c>
-      <c r="D43" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E43" s="25" t="n"/>
+      <c r="D43" s="38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E43" s="39" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
@@ -2753,7 +2753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -3140,6 +3140,22 @@
         <v>800</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>#803 Steve (拿聖代冰淇淋款)
+#922 Robin (拿白板款)</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="n">
+        <v>800</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 881 and 427 as sold for 1600 and add reservation notes to Excel
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -136,6 +136,27 @@
     </font>
     <font>
       <name val="微軟正黑體"/>
+      <charset val="136"/>
+      <family val="2"/>
+      <strike val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <charset val="136"/>
+      <family val="2"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <charset val="136"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
       <strike val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
@@ -144,14 +165,8 @@
       <name val="微軟正黑體"/>
       <sz val="12"/>
     </font>
-    <font>
-      <name val="微軟正黑體"/>
-      <strike val="0"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="21">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -244,8 +259,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCC0DA"/>
+        <bgColor rgb="FFCCC0DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -266,19 +305,28 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-        <bgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -359,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -392,7 +440,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -485,6 +532,18 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -859,8 +918,8 @@
     <col width="79.87890625" customWidth="1" style="2" min="3" max="3"/>
     <col width="16.5859375" customWidth="1" style="2" min="4" max="4"/>
     <col width="23.76171875" customWidth="1" style="3" min="5" max="5"/>
-    <col width="8.9375" customWidth="1" style="2" min="6" max="13"/>
-    <col width="8.9375" customWidth="1" style="2" min="14" max="16384"/>
+    <col width="8.9375" customWidth="1" style="2" min="6" max="14"/>
+    <col width="8.9375" customWidth="1" style="2" min="15" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.3" customHeight="1">
@@ -891,1856 +950,1856 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>8-Bit</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Stranger Things 8-Bit 4-Pack (像素復古四入組)</t>
         </is>
       </c>
-      <c r="D2" s="21" t="n">
+      <c r="D2" s="20" t="n">
         <v>1750</v>
       </c>
-      <c r="E2" s="22" t="n"/>
+      <c r="E2" s="21" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Town #50</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>Rockin' Robin with The Squawk (廣播站建築組)</t>
         </is>
       </c>
-      <c r="D3" s="21" t="n">
+      <c r="D3" s="20" t="n">
         <v>1000</v>
       </c>
-      <c r="E3" s="22" t="n"/>
+      <c r="E3" s="21" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Rides #137</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Steve Harrington (經典車輛組)</t>
         </is>
       </c>
-      <c r="D4" s="21" t="n">
+      <c r="D4" s="20" t="n">
         <v>1500</v>
       </c>
-      <c r="E4" s="22" t="n"/>
+      <c r="E4" s="21" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Rides #138</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Steve with The Squawk Van (廣播箱型車)</t>
         </is>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="20" t="n">
         <v>1500</v>
       </c>
-      <c r="E5" s="22" t="n"/>
+      <c r="E5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>#421</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Eleven with Eggos (Chase 稀有金髮版)</t>
         </is>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="E6" s="17" t="n"/>
+      <c r="E6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>#423</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Mike (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="17" t="n">
         <v>850</v>
       </c>
-      <c r="E7" s="19" t="n"/>
+      <c r="E7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>#424</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>Dustin (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="17" t="n">
         <v>850</v>
       </c>
-      <c r="E8" s="19" t="n"/>
+      <c r="E8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>#425</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>Lucas (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="23" t="n">
         <v>850</v>
       </c>
-      <c r="E9" s="25" t="n"/>
+      <c r="E9" s="24" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>#426</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Will (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="17" t="n">
         <v>850</v>
       </c>
-      <c r="E10" s="19" t="n"/>
+      <c r="E10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="A11" s="43" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>#427</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>Barb (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="43" t="n">
         <v>700</v>
       </c>
-      <c r="E11" s="25" t="n"/>
+      <c r="E11" s="44" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
         <is>
           <t>#428</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="C12" s="37" t="inlineStr">
         <is>
           <t>Demogorgon (魔王開口款)</t>
         </is>
       </c>
-      <c r="D12" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E12" s="39" t="n"/>
+      <c r="D12" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E12" s="38" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B13" s="31" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>#436</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>Joyce (第一季聖誕燈泡)</t>
         </is>
       </c>
-      <c r="D13" s="31" t="n">
-        <v>500</v>
-      </c>
-      <c r="E13" s="32" t="n"/>
+      <c r="D13" s="30" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" s="31" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B14" s="38" t="inlineStr">
+      <c r="B14" s="37" t="inlineStr">
         <is>
           <t>#476</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="C14" s="37" t="inlineStr">
         <is>
           <t>Mr. Clarke (2017 SDCC 展會限定)</t>
         </is>
       </c>
-      <c r="D14" s="38" t="n">
+      <c r="D14" s="37" t="n">
         <v>1500</v>
       </c>
-      <c r="E14" s="39" t="n"/>
+      <c r="E14" s="38" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
         <is>
           <t>#512</t>
         </is>
       </c>
-      <c r="C15" s="38" t="inlineStr">
+      <c r="C15" s="37" t="inlineStr">
         <is>
           <t>Hopper (警長常規款)</t>
         </is>
       </c>
-      <c r="D15" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E15" s="39" t="n"/>
+      <c r="D15" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E15" s="38" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B16" s="38" t="inlineStr">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
         <is>
           <t>#513</t>
         </is>
       </c>
-      <c r="C16" s="38" t="inlineStr">
+      <c r="C16" s="37" t="inlineStr">
         <is>
           <t>Jonathan (第一季照相機)</t>
         </is>
       </c>
-      <c r="D16" s="38" t="n">
+      <c r="D16" s="37" t="n">
         <v>750</v>
       </c>
-      <c r="E16" s="39" t="n"/>
+      <c r="E16" s="38" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B17" s="38" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>#514</t>
         </is>
       </c>
-      <c r="C17" s="38" t="inlineStr">
+      <c r="C17" s="37" t="inlineStr">
         <is>
           <t>Nancy (第一季拿槍款)</t>
         </is>
       </c>
-      <c r="D17" s="38" t="n">
+      <c r="D17" s="37" t="n">
         <v>750</v>
       </c>
-      <c r="E17" s="39" t="n"/>
+      <c r="E17" s="38" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B18" s="38" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
         <is>
           <t>#515</t>
         </is>
       </c>
-      <c r="C18" s="38" t="inlineStr">
+      <c r="C18" s="37" t="inlineStr">
         <is>
           <t>Brenner (布倫納博士)</t>
         </is>
       </c>
-      <c r="D18" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E18" s="39" t="n"/>
+      <c r="D18" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E18" s="38" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>#545</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>Eleven (實驗室病人服)</t>
         </is>
       </c>
-      <c r="D19" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E19" s="25" t="n"/>
+      <c r="D19" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E19" s="24" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B20" s="38" t="inlineStr">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
         <is>
           <t>#550</t>
         </is>
       </c>
-      <c r="C20" s="38" t="inlineStr">
+      <c r="C20" s="37" t="inlineStr">
         <is>
           <t>Joyce (磁鐵版)</t>
         </is>
       </c>
-      <c r="D20" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E20" s="39" t="n"/>
+      <c r="D20" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E20" s="38" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B21" s="38" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>#572</t>
         </is>
       </c>
-      <c r="C21" s="38" t="inlineStr">
+      <c r="C21" s="37" t="inlineStr">
         <is>
           <t>Eleven (BoxLunch 限定 吊帶褲)</t>
         </is>
       </c>
-      <c r="D21" s="38" t="inlineStr">
+      <c r="D21" s="37" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="E21" s="39" t="n"/>
+      <c r="E21" s="38" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>#593</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>Dustin &amp; Dart (Hot Topic 限定)</t>
         </is>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="17" t="n">
         <v>750</v>
       </c>
-      <c r="E22" s="19" t="n"/>
+      <c r="E22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>#637</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr">
+      <c r="C23" s="37" t="inlineStr">
         <is>
           <t>Eleven (Elevated 升空施法)</t>
         </is>
       </c>
-      <c r="D23" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E23" s="39" t="n"/>
+      <c r="D23" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E23" s="38" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>🎲 常規小盒</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>#638</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>Steve (經典款)</t>
         </is>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="17" t="n">
         <v>800</v>
       </c>
-      <c r="E24" s="19" t="n"/>
+      <c r="E24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B25" s="38" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>#640</t>
         </is>
       </c>
-      <c r="C25" s="38" t="inlineStr">
+      <c r="C25" s="37" t="inlineStr">
         <is>
           <t>Billy (比利經典款)</t>
         </is>
       </c>
-      <c r="D25" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E25" s="39" t="n"/>
+      <c r="D25" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E25" s="38" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B26" s="38" t="inlineStr">
+      <c r="A26" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B26" s="37" t="inlineStr">
         <is>
           <t>#643</t>
         </is>
       </c>
-      <c r="C26" s="38" t="inlineStr">
+      <c r="C26" s="37" t="inlineStr">
         <is>
           <t>Vampire Bob (吸血鬼鮑伯)</t>
         </is>
       </c>
-      <c r="D26" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E26" s="39" t="n"/>
+      <c r="D26" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E26" s="38" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B27" s="31" t="inlineStr">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>#674</t>
         </is>
       </c>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="C27" s="30" t="inlineStr">
         <is>
           <t>Robin (冰淇淋制服款)</t>
         </is>
       </c>
-      <c r="D27" s="31" t="n">
-        <v>500</v>
-      </c>
-      <c r="E27" s="32" t="n"/>
+      <c r="D27" s="30" t="n">
+        <v>500</v>
+      </c>
+      <c r="E27" s="31" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B28" s="31" t="inlineStr">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
         <is>
           <t>#675</t>
         </is>
       </c>
-      <c r="C28" s="31" t="inlineStr">
+      <c r="C28" s="30" t="inlineStr">
         <is>
           <t>Steve (SDCC 限定)</t>
         </is>
       </c>
-      <c r="D28" s="31" t="n">
+      <c r="D28" s="30" t="n">
         <v>750</v>
       </c>
-      <c r="E28" s="32" t="n"/>
+      <c r="E28" s="31" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>#717</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>Eleven (雪球舞會洋裝)</t>
         </is>
       </c>
-      <c r="D29" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E29" s="19" t="n"/>
+      <c r="D29" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="42" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B30" s="42" t="inlineStr">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B30" s="41" t="inlineStr">
         <is>
           <t>#720</t>
         </is>
       </c>
-      <c r="C30" s="42" t="inlineStr">
+      <c r="C30" s="41" t="inlineStr">
         <is>
           <t>Hopper (約會襯衫款)</t>
         </is>
       </c>
-      <c r="D30" s="42" t="n">
-        <v>500</v>
-      </c>
-      <c r="E30" s="43" t="n"/>
+      <c r="D30" s="41" t="n">
+        <v>500</v>
+      </c>
+      <c r="E30" s="42" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Moments #727</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C31" s="19" t="inlineStr">
         <is>
           <t>Eleven and Demogorgon (11號對決魔王名場面) (戰鬥名場面2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D31" s="21" t="n">
+      <c r="D31" s="20" t="n">
         <v>2000</v>
       </c>
-      <c r="E31" s="22" t="n"/>
+      <c r="E31" s="21" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Moments #728</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C32" s="19" t="inlineStr">
         <is>
           <t>Steve and Demodog (史帝夫對決魔犬名場面) (戰鬥名場面2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D32" s="21" t="n">
+      <c r="D32" s="20" t="n">
         <v>2000</v>
       </c>
-      <c r="E32" s="22" t="n"/>
+      <c r="E32" s="21" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>#729</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
         <is>
           <t>Mike (雪球舞會西裝)</t>
         </is>
       </c>
-      <c r="D33" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E33" s="19" t="n"/>
+      <c r="D33" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E33" s="18" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B34" s="38" t="inlineStr">
+      <c r="A34" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B34" s="37" t="inlineStr">
         <is>
           <t>#803</t>
         </is>
       </c>
-      <c r="C34" s="38" t="inlineStr">
+      <c r="C34" s="37" t="inlineStr">
         <is>
           <t>Steve (拿聖代冰淇淋款)</t>
         </is>
       </c>
-      <c r="D34" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E34" s="39" t="n"/>
+      <c r="D34" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E34" s="38" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B35" s="38" t="inlineStr">
+      <c r="A35" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B35" s="37" t="inlineStr">
         <is>
           <t>#804</t>
         </is>
       </c>
-      <c r="C35" s="38" t="inlineStr">
+      <c r="C35" s="37" t="inlineStr">
         <is>
           <t>Dustin (Walmart 限定 夏令營帽子)</t>
         </is>
       </c>
-      <c r="D35" s="38" t="n">
+      <c r="D35" s="37" t="n">
         <v>650</v>
       </c>
-      <c r="E35" s="39" t="n"/>
+      <c r="E35" s="38" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="inlineStr">
         <is>
           <t>#807</t>
         </is>
       </c>
-      <c r="C36" s="23" t="inlineStr">
+      <c r="C36" s="22" t="inlineStr">
         <is>
           <t>Lucas (S3 商場造型)</t>
         </is>
       </c>
-      <c r="D36" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E36" s="25" t="n"/>
+      <c r="D36" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E36" s="24" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
         <is>
           <t>#808</t>
         </is>
       </c>
-      <c r="C37" s="23" t="inlineStr">
+      <c r="C37" s="22" t="inlineStr">
         <is>
           <t>Erica (經典款)</t>
         </is>
       </c>
-      <c r="D37" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E37" s="25" t="n"/>
+      <c r="D37" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E37" s="24" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B38" s="23" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>#826</t>
         </is>
       </c>
-      <c r="C38" s="23" t="inlineStr">
+      <c r="C38" s="22" t="inlineStr">
         <is>
           <t>Battle Eleven (商場大戰眼罩款)</t>
         </is>
       </c>
-      <c r="D38" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E38" s="25" t="n"/>
+      <c r="D38" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E38" s="24" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B39" s="23" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>#827</t>
         </is>
       </c>
-      <c r="C39" s="23" t="inlineStr">
+      <c r="C39" s="22" t="inlineStr">
         <is>
           <t>Eleven (紅色外套)</t>
         </is>
       </c>
-      <c r="D39" s="24" t="inlineStr">
+      <c r="D39" s="23" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="E39" s="25" t="n"/>
+      <c r="E39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B40" s="18" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>#828</t>
         </is>
       </c>
-      <c r="C40" s="18" t="inlineStr">
+      <c r="C40" s="17" t="inlineStr">
         <is>
           <t>Dustin (Target 烤牛肉 T-shirt)</t>
         </is>
       </c>
-      <c r="D40" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E40" s="19" t="n"/>
+      <c r="D40" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E40" s="18" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B41" s="23" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
         <is>
           <t>#843</t>
         </is>
       </c>
-      <c r="C41" s="23" t="inlineStr">
+      <c r="C41" s="22" t="inlineStr">
         <is>
           <t>Eleven (黑色幾何圖騰洋裝)</t>
         </is>
       </c>
-      <c r="D41" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E41" s="25" t="n"/>
+      <c r="D41" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E41" s="24" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="inlineStr">
+      <c r="A42" s="43" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B42" s="43" t="inlineStr">
         <is>
           <t>#881</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C42" s="43" t="inlineStr">
         <is>
           <t>Suzie (2019 NYCC 展會限定)</t>
         </is>
       </c>
-      <c r="D42" s="16" t="n">
+      <c r="D42" s="43" t="n">
         <v>1300</v>
       </c>
-      <c r="E42" s="17" t="n"/>
+      <c r="E42" s="44" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B43" s="38" t="inlineStr">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B43" s="37" t="inlineStr">
         <is>
           <t>#922</t>
         </is>
       </c>
-      <c r="C43" s="38" t="inlineStr">
+      <c r="C43" s="37" t="inlineStr">
         <is>
           <t>Robin (拿白板款)</t>
         </is>
       </c>
-      <c r="D43" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E43" s="39" t="n"/>
+      <c r="D43" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E43" s="38" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="38" t="inlineStr">
+      <c r="A44" s="37" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B44" s="38" t="inlineStr">
+      <c r="B44" s="37" t="inlineStr">
         <is>
           <t>Deluxe #1186</t>
         </is>
       </c>
-      <c r="C44" s="38" t="inlineStr">
+      <c r="C44" s="37" t="inlineStr">
         <is>
           <t>Byers House: Demogorgon (拜爾斯家魔王破牆)</t>
         </is>
       </c>
-      <c r="D44" s="38" t="n">
+      <c r="D44" s="37" t="n">
         <v>1000</v>
       </c>
-      <c r="E44" s="39" t="n"/>
+      <c r="E44" s="38" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="28" t="inlineStr">
+      <c r="A45" s="27" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B45" s="28" t="inlineStr">
+      <c r="B45" s="27" t="inlineStr">
         <is>
           <t>Deluxe #1187</t>
         </is>
       </c>
-      <c r="C45" s="28" t="inlineStr">
+      <c r="C45" s="27" t="inlineStr">
         <is>
           <t>Byers House: Will (拜爾斯家威爾與燈牆)</t>
         </is>
       </c>
-      <c r="D45" s="29" t="n">
+      <c r="D45" s="28" t="n">
         <v>1000</v>
       </c>
-      <c r="E45" s="30" t="n"/>
+      <c r="E45" s="29" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B46" s="23" t="inlineStr">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>#1241</t>
         </is>
       </c>
-      <c r="C46" s="23" t="inlineStr">
+      <c r="C46" s="22" t="inlineStr">
         <is>
           <t>Lucas (S4 籃球隊服)</t>
         </is>
       </c>
-      <c r="D46" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E46" s="25" t="n"/>
+      <c r="D46" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E46" s="24" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>#1250</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
         <is>
           <t>Eddie (Target 限定 黑光版)</t>
         </is>
       </c>
-      <c r="D47" s="16" t="n">
+      <c r="D47" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="E47" s="17" t="n"/>
+      <c r="E47" s="16" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="38" t="inlineStr">
+      <c r="A48" s="37" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B48" s="38" t="inlineStr">
+      <c r="B48" s="37" t="inlineStr">
         <is>
           <t>#1250</t>
         </is>
       </c>
-      <c r="C48" s="38" t="inlineStr">
+      <c r="C48" s="37" t="inlineStr">
         <is>
           <t>Eddie (Target 限定 經典吉他版)</t>
         </is>
       </c>
-      <c r="D48" s="38" t="n">
+      <c r="D48" s="37" t="n">
         <v>800</v>
       </c>
-      <c r="E48" s="39" t="n"/>
+      <c r="E48" s="38" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
         <is>
           <t>#1297</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="C49" s="17" t="inlineStr">
         <is>
           <t>Eleven (彩虹室病人服)</t>
         </is>
       </c>
-      <c r="D49" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E49" s="19" t="n"/>
+      <c r="D49" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E49" s="18" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B50" s="38" t="inlineStr">
+      <c r="A50" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B50" s="37" t="inlineStr">
         <is>
           <t>#1301</t>
         </is>
       </c>
-      <c r="C50" s="38" t="inlineStr">
+      <c r="C50" s="37" t="inlineStr">
         <is>
           <t>Erica (S4 戰鬥裝備)</t>
         </is>
       </c>
-      <c r="D50" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E50" s="39" t="n"/>
+      <c r="D50" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E50" s="38" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
         <is>
           <t>#1303</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C51" s="17" t="inlineStr">
         <is>
           <t>Demobat (顛倒世界魔蝠)</t>
         </is>
       </c>
-      <c r="D51" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E51" s="19" t="n"/>
+      <c r="D51" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E51" s="18" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B52" s="18" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
         <is>
           <t>#1312</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
+      <c r="C52" s="17" t="inlineStr">
         <is>
           <t>Vecna (Black Light 黑光版)</t>
         </is>
       </c>
-      <c r="D52" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E52" s="19" t="n"/>
+      <c r="D52" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E52" s="18" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B53" s="23" t="inlineStr">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>#1457</t>
         </is>
       </c>
-      <c r="C53" s="23" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>Eleven (S4 流鼻血戰鬥款)</t>
         </is>
       </c>
-      <c r="D53" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E53" s="25" t="n"/>
+      <c r="D53" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E53" s="24" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B54" s="23" t="inlineStr">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>#1459</t>
         </is>
       </c>
-      <c r="C54" s="23" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>Jonathan (S4 經典款)</t>
         </is>
       </c>
-      <c r="D54" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E54" s="25" t="n"/>
+      <c r="D54" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E54" s="24" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B55" s="23" t="inlineStr">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>#1461</t>
         </is>
       </c>
-      <c r="C55" s="23" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>Robin (貝雷帽款式)</t>
         </is>
       </c>
-      <c r="D55" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E55" s="25" t="n"/>
+      <c r="D55" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E55" s="24" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B56" s="38" t="inlineStr">
+      <c r="A56" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B56" s="37" t="inlineStr">
         <is>
           <t>#1462</t>
         </is>
       </c>
-      <c r="C56" s="38" t="inlineStr">
+      <c r="C56" s="37" t="inlineStr">
         <is>
           <t>Eddie (Special Edition 顛倒世界戰鬥 - 有貼紙)</t>
         </is>
       </c>
-      <c r="D56" s="38" t="n">
+      <c r="D56" s="37" t="n">
         <v>800</v>
       </c>
-      <c r="E56" s="39" t="n"/>
+      <c r="E56" s="38" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="18" t="inlineStr">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>🎲 常規小盒</t>
         </is>
       </c>
-      <c r="B57" s="18" t="inlineStr">
+      <c r="B57" s="17" t="inlineStr">
         <is>
           <t>#1462</t>
         </is>
       </c>
-      <c r="C57" s="18" t="inlineStr">
+      <c r="C57" s="17" t="inlineStr">
         <is>
           <t>Eddie (Special Edition 顛倒世界戰鬥 - 無貼紙)</t>
         </is>
       </c>
-      <c r="D57" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E57" s="19" t="n"/>
+      <c r="D57" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E57" s="18" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="31" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B58" s="31" t="inlineStr">
+      <c r="A58" s="30" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B58" s="30" t="inlineStr">
         <is>
           <t>#1463</t>
         </is>
       </c>
-      <c r="C58" s="31" t="inlineStr">
+      <c r="C58" s="30" t="inlineStr">
         <is>
           <t>Dustin (地獄火盾牌長矛)</t>
         </is>
       </c>
-      <c r="D58" s="31" t="n">
-        <v>500</v>
-      </c>
-      <c r="E58" s="32" t="n"/>
+      <c r="D58" s="30" t="n">
+        <v>500</v>
+      </c>
+      <c r="E58" s="31" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B59" s="23" t="inlineStr">
+      <c r="A59" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B59" s="22" t="inlineStr">
         <is>
           <t>#1538</t>
         </is>
       </c>
-      <c r="C59" s="23" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>Chrissy (啦啦隊長)</t>
         </is>
       </c>
-      <c r="D59" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E59" s="25" t="n"/>
+      <c r="D59" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E59" s="24" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B60" s="23" t="inlineStr">
+      <c r="A60" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B60" s="22" t="inlineStr">
         <is>
           <t>#1540</t>
         </is>
       </c>
-      <c r="C60" s="23" t="inlineStr">
+      <c r="C60" s="22" t="inlineStr">
         <is>
           <t>Vecna (S4 常規款)</t>
         </is>
       </c>
-      <c r="D60" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E60" s="25" t="n"/>
+      <c r="D60" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E60" s="24" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B61" s="23" t="inlineStr">
+      <c r="A61" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B61" s="22" t="inlineStr">
         <is>
           <t>#1542</t>
         </is>
       </c>
-      <c r="C61" s="23" t="inlineStr">
+      <c r="C61" s="22" t="inlineStr">
         <is>
           <t>Steve (顛倒世界拿手電筒)</t>
         </is>
       </c>
-      <c r="D61" s="24" t="n">
+      <c r="D61" s="23" t="n">
         <v>800</v>
       </c>
-      <c r="E61" s="25" t="n"/>
+      <c r="E61" s="24" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B62" s="23" t="inlineStr">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B62" s="22" t="inlineStr">
         <is>
           <t>#1543</t>
         </is>
       </c>
-      <c r="C62" s="23" t="inlineStr">
+      <c r="C62" s="22" t="inlineStr">
         <is>
           <t>Murray (火焰噴射器)</t>
         </is>
       </c>
-      <c r="D62" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E62" s="25" t="n"/>
+      <c r="D62" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E62" s="24" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B63" s="23" t="inlineStr">
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B63" s="22" t="inlineStr">
         <is>
           <t>#1545</t>
         </is>
       </c>
-      <c r="C63" s="23" t="inlineStr">
+      <c r="C63" s="22" t="inlineStr">
         <is>
           <t>Steve (Scoops Ahoy 復古包裝)</t>
         </is>
       </c>
-      <c r="D63" s="24" t="n">
+      <c r="D63" s="23" t="n">
         <v>750</v>
       </c>
-      <c r="E63" s="25" t="n"/>
+      <c r="E63" s="24" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B64" s="23" t="inlineStr">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B64" s="22" t="inlineStr">
         <is>
           <t>#1546</t>
         </is>
       </c>
-      <c r="C64" s="23" t="inlineStr">
+      <c r="C64" s="22" t="inlineStr">
         <is>
           <t>Robin (Scoops Ahoy 復古包裝)</t>
         </is>
       </c>
-      <c r="D64" s="24" t="n">
+      <c r="D64" s="23" t="n">
         <v>750</v>
       </c>
-      <c r="E64" s="25" t="n"/>
+      <c r="E64" s="24" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B65" s="18" t="inlineStr">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
         <is>
           <t>#1547</t>
         </is>
       </c>
-      <c r="C65" s="18" t="inlineStr">
+      <c r="C65" s="17" t="inlineStr">
         <is>
           <t>Demogorgon (Scoops Ahoy 冰淇淋魔王)</t>
         </is>
       </c>
-      <c r="D65" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E65" s="19" t="n"/>
+      <c r="D65" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E65" s="18" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B66" s="23" t="inlineStr">
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B66" s="22" t="inlineStr">
         <is>
           <t>#1559</t>
         </is>
       </c>
-      <c r="C66" s="23" t="inlineStr">
+      <c r="C66" s="22" t="inlineStr">
         <is>
           <t>001 Vaporizing (2024 SDCC 消散版) (有2隻)</t>
         </is>
       </c>
-      <c r="D66" s="24" t="n">
+      <c r="D66" s="23" t="n">
         <v>700</v>
       </c>
-      <c r="E66" s="25" t="n"/>
+      <c r="E66" s="24" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="26" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B67" s="26" t="inlineStr">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B67" s="25" t="inlineStr">
         <is>
           <t>#1595</t>
         </is>
       </c>
-      <c r="C67" s="26" t="inlineStr">
+      <c r="C67" s="25" t="inlineStr">
         <is>
           <t>Vecna</t>
         </is>
       </c>
-      <c r="D67" s="27" t="n">
+      <c r="D67" s="26" t="n">
         <v>700</v>
       </c>
-      <c r="E67" s="25" t="n"/>
+      <c r="E67" s="24" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="26" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B68" s="26" t="inlineStr">
+      <c r="A68" s="25" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B68" s="25" t="inlineStr">
         <is>
           <t>#1596</t>
         </is>
       </c>
-      <c r="C68" s="26" t="inlineStr">
+      <c r="C68" s="25" t="inlineStr">
         <is>
           <t>Demogorgon</t>
         </is>
       </c>
-      <c r="D68" s="27" t="n">
+      <c r="D68" s="26" t="n">
         <v>700</v>
       </c>
-      <c r="E68" s="25" t="n"/>
+      <c r="E68" s="24" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="20" t="inlineStr">
+      <c r="A69" s="19" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B69" s="20" t="inlineStr">
+      <c r="B69" s="19" t="inlineStr">
         <is>
           <t>#1597</t>
         </is>
       </c>
-      <c r="C69" s="20" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>The Mind Flayer (超大盒 奪心魔) (輕微盒損)</t>
         </is>
       </c>
-      <c r="D69" s="21" t="n">
+      <c r="D69" s="20" t="n">
         <v>400</v>
       </c>
-      <c r="E69" s="22" t="n"/>
+      <c r="E69" s="21" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B70" s="38" t="inlineStr">
+      <c r="A70" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B70" s="37" t="inlineStr">
         <is>
           <t>#1778</t>
         </is>
       </c>
-      <c r="C70" s="38" t="inlineStr">
+      <c r="C70" s="37" t="inlineStr">
         <is>
           <t>Nancy Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D70" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E70" s="39" t="n"/>
+      <c r="D70" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E70" s="38" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B71" s="38" t="inlineStr">
+      <c r="A71" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B71" s="37" t="inlineStr">
         <is>
           <t>#1780</t>
         </is>
       </c>
-      <c r="C71" s="38" t="inlineStr">
+      <c r="C71" s="37" t="inlineStr">
         <is>
           <t>Eleven (Season 5)</t>
         </is>
       </c>
-      <c r="D71" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E71" s="39" t="n"/>
+      <c r="D71" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E71" s="38" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B72" s="23" t="inlineStr">
+      <c r="A72" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B72" s="22" t="inlineStr">
         <is>
           <t>#1781</t>
         </is>
       </c>
-      <c r="C72" s="23" t="inlineStr">
+      <c r="C72" s="22" t="inlineStr">
         <is>
           <t>Dustin Henderson (Season 5)</t>
         </is>
       </c>
-      <c r="D72" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E72" s="25" t="n"/>
+      <c r="D72" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E72" s="24" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B73" s="38" t="inlineStr">
+      <c r="A73" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B73" s="37" t="inlineStr">
         <is>
           <t>#1782</t>
         </is>
       </c>
-      <c r="C73" s="38" t="inlineStr">
+      <c r="C73" s="37" t="inlineStr">
         <is>
           <t>Holly Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D73" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E73" s="39" t="n"/>
+      <c r="D73" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E73" s="38" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B74" s="38" t="inlineStr">
+      <c r="A74" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B74" s="37" t="inlineStr">
         <is>
           <t>#1783</t>
         </is>
       </c>
-      <c r="C74" s="38" t="inlineStr">
+      <c r="C74" s="37" t="inlineStr">
         <is>
           <t>Mike Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D74" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E74" s="39" t="n"/>
+      <c r="D74" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E74" s="38" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B75" s="23" t="inlineStr">
+      <c r="A75" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B75" s="22" t="inlineStr">
         <is>
           <t>#1784</t>
         </is>
       </c>
-      <c r="C75" s="23" t="inlineStr">
+      <c r="C75" s="22" t="inlineStr">
         <is>
           <t>Jim Hopper (Season 5)</t>
         </is>
       </c>
-      <c r="D75" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E75" s="25" t="n"/>
+      <c r="D75" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E75" s="24" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B76" s="23" t="inlineStr">
+      <c r="A76" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B76" s="22" t="inlineStr">
         <is>
           <t>#1785</t>
         </is>
       </c>
-      <c r="C76" s="23" t="inlineStr">
+      <c r="C76" s="22" t="inlineStr">
         <is>
           <t>Lucas Sinclair (Season 5)</t>
         </is>
       </c>
-      <c r="D76" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E76" s="25" t="n"/>
+      <c r="D76" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E76" s="24" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B77" s="18" t="inlineStr">
+      <c r="A77" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="inlineStr">
         <is>
           <t>#1786</t>
         </is>
       </c>
-      <c r="C77" s="18" t="inlineStr">
+      <c r="C77" s="17" t="inlineStr">
         <is>
           <t>Will Byers (Season 5)</t>
         </is>
       </c>
-      <c r="D77" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E77" s="19" t="n"/>
+      <c r="D77" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E77" s="18" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="18" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B78" s="18" t="inlineStr">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="inlineStr">
         <is>
           <t>#1796</t>
         </is>
       </c>
-      <c r="C78" s="18" t="inlineStr">
+      <c r="C78" s="17" t="inlineStr">
         <is>
           <t>Dustin Henderson (Season 5)</t>
         </is>
       </c>
-      <c r="D78" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="E78" s="19" t="n"/>
+      <c r="D78" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E78" s="18" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B79" s="38" t="inlineStr">
+      <c r="A79" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B79" s="37" t="inlineStr">
         <is>
           <t>#1797</t>
         </is>
       </c>
-      <c r="C79" s="38" t="inlineStr">
+      <c r="C79" s="37" t="inlineStr">
         <is>
           <t>Jonathan Byers (Season 5)</t>
         </is>
       </c>
-      <c r="D79" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E79" s="39" t="n"/>
+      <c r="D79" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E79" s="38" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B80" s="38" t="inlineStr">
+      <c r="A80" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B80" s="37" t="inlineStr">
         <is>
           <t>#1798</t>
         </is>
       </c>
-      <c r="C80" s="38" t="inlineStr">
+      <c r="C80" s="37" t="inlineStr">
         <is>
           <t>Lucas Sinclair (S5 WSQK 特別款)</t>
         </is>
       </c>
-      <c r="D80" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E80" s="39" t="n"/>
+      <c r="D80" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E80" s="38" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B81" s="38" t="inlineStr">
+      <c r="A81" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B81" s="37" t="inlineStr">
         <is>
           <t>#1802</t>
         </is>
       </c>
-      <c r="C81" s="38" t="inlineStr">
+      <c r="C81" s="37" t="inlineStr">
         <is>
           <t>Nancy Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D81" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E81" s="39" t="n"/>
+      <c r="D81" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E81" s="38" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B82" s="23" t="inlineStr">
+      <c r="A82" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B82" s="22" t="inlineStr">
         <is>
           <t>#1805</t>
         </is>
       </c>
-      <c r="C82" s="23" t="inlineStr">
+      <c r="C82" s="22" t="inlineStr">
         <is>
           <t>Max Mayfield (Season 5)</t>
         </is>
       </c>
-      <c r="D82" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E82" s="25" t="n"/>
+      <c r="D82" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E82" s="24" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B83" s="23" t="inlineStr">
+      <c r="A83" s="22" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B83" s="22" t="inlineStr">
         <is>
           <t>#1807</t>
         </is>
       </c>
-      <c r="C83" s="23" t="inlineStr">
+      <c r="C83" s="22" t="inlineStr">
         <is>
           <t>Eleven (Season 5)</t>
         </is>
       </c>
-      <c r="D83" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E83" s="25" t="n"/>
+      <c r="D83" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E83" s="24" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B84" s="38" t="inlineStr">
+      <c r="A84" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B84" s="37" t="inlineStr">
         <is>
           <t>#1808</t>
         </is>
       </c>
-      <c r="C84" s="38" t="inlineStr">
+      <c r="C84" s="37" t="inlineStr">
         <is>
           <t>Mr. Whatsit (Season 5)</t>
         </is>
       </c>
-      <c r="D84" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E84" s="39" t="n"/>
+      <c r="D84" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E84" s="38" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="38" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B85" s="38" t="inlineStr">
+      <c r="A85" s="37" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B85" s="37" t="inlineStr">
         <is>
           <t>#1810</t>
         </is>
       </c>
-      <c r="C85" s="38" t="inlineStr">
+      <c r="C85" s="37" t="inlineStr">
         <is>
           <t>Holly The Heroic (S5 英雄霍莉)</t>
         </is>
       </c>
-      <c r="D85" s="38" t="n">
-        <v>500</v>
-      </c>
-      <c r="E85" s="39" t="n"/>
+      <c r="D85" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E85" s="38" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="35" t="inlineStr">
+      <c r="A86" s="34" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B86" s="35" t="inlineStr">
+      <c r="B86" s="34" t="inlineStr">
         <is>
           <t>#1831</t>
         </is>
       </c>
-      <c r="C86" s="35" t="inlineStr">
+      <c r="C86" s="34" t="inlineStr">
         <is>
           <t>Demogorgon (S5 最新魔王款)</t>
         </is>
       </c>
-      <c r="D86" s="36" t="n">
+      <c r="D86" s="35" t="n">
         <v>1200</v>
       </c>
-      <c r="E86" s="37" t="n"/>
+      <c r="E86" s="36" t="n"/>
     </row>
     <row r="87" ht="15.3" customHeight="1">
-      <c r="A87" s="38" t="inlineStr">
+      <c r="A87" s="37" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B87" s="38" t="inlineStr">
+      <c r="B87" s="37" t="inlineStr">
         <is>
           <t>套組</t>
         </is>
       </c>
-      <c r="C87" s="38" t="inlineStr">
+      <c r="C87" s="37" t="inlineStr">
         <is>
           <t>捉鬼敢死隊 4 人組 (#546, #547, #548, #549)</t>
         </is>
       </c>
-      <c r="D87" s="38" t="n">
+      <c r="D87" s="37" t="n">
         <v>3700</v>
       </c>
-      <c r="E87" s="39" t="n"/>
+      <c r="E87" s="38" t="n"/>
     </row>
     <row r="88" ht="15.3" customHeight="1">
-      <c r="A88" s="15" t="inlineStr">
+      <c r="A88" s="14" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B88" s="15" t="inlineStr">
+      <c r="B88" s="14" t="inlineStr">
         <is>
           <t>套組</t>
         </is>
       </c>
-      <c r="C88" s="15" t="inlineStr">
+      <c r="C88" s="14" t="inlineStr">
         <is>
           <t>Robin &amp; Steve 2-Pack (Blacklight 黑光版雙入組)</t>
         </is>
       </c>
-      <c r="D88" s="16" t="n">
+      <c r="D88" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="E88" s="17" t="n"/>
+      <c r="E88" s="16" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="38" t="inlineStr">
+      <c r="A89" s="37" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B89" s="38" t="inlineStr">
+      <c r="B89" s="37" t="inlineStr">
         <is>
           <t>套組</t>
         </is>
       </c>
-      <c r="C89" s="38" t="inlineStr">
+      <c r="C89" s="37" t="inlineStr">
         <is>
           <t>Vecna &amp; Vecna 雙入組 (2022 NYCC 展會限定)</t>
         </is>
       </c>
-      <c r="D89" s="38" t="n">
+      <c r="D89" s="37" t="n">
         <v>900</v>
       </c>
-      <c r="E89" s="39" t="n"/>
+      <c r="E89" s="38" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2753,7 +2812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -2761,8 +2820,8 @@
     <col width="20" customWidth="1" style="2" min="3" max="3"/>
     <col width="8.9375" customWidth="1" style="2" min="4" max="5"/>
     <col width="8.9375" customWidth="1" style="8" min="6" max="6"/>
-    <col width="8.9375" customWidth="1" style="2" min="7" max="10"/>
-    <col width="8.9375" customWidth="1" style="2" min="11" max="16384"/>
+    <col width="8.9375" customWidth="1" style="2" min="7" max="11"/>
+    <col width="8.9375" customWidth="1" style="2" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.3" customHeight="1">
@@ -2892,6 +2951,7 @@
       <c r="C7" s="5" t="n">
         <v>1000</v>
       </c>
+      <c r="F7" s="2" t="n"/>
     </row>
     <row r="8" ht="198.9" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
@@ -2914,9 +2974,7 @@
       <c r="C8" s="11" t="n">
         <v>5000</v>
       </c>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
+      <c r="F8" s="2" t="n"/>
     </row>
     <row r="9" ht="61.2" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -2932,9 +2990,7 @@
       <c r="C9" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
+      <c r="F9" s="2" t="n"/>
     </row>
     <row r="10" ht="15.3" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -2950,32 +3006,31 @@
       <c r="C10" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
+      <c r="F10" s="2" t="n"/>
     </row>
     <row r="11" ht="15.3" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>#1805 Max Mayfield (Season 5)</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>500</v>
-      </c>
+      <c r="C11" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="F11" s="2" t="n"/>
     </row>
     <row r="12" ht="61.2" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B12" s="34" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>#436 Joyce (第一季聖誕燈泡)
 #674 Robin (冰淇淋制服款)
@@ -2983,64 +3038,65 @@
 #1463 Dustin (地獄火盾牌長矛)</t>
         </is>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C12" s="33" t="n">
         <v>2100</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="40" t="inlineStr">
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="15.3" customHeight="1">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="B13" s="41" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>#1808 Mr. Whatsit (Season 5)</t>
         </is>
       </c>
-      <c r="C13" s="41" t="n">
+      <c r="C13" s="40" t="n">
         <v>400</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="40" t="inlineStr">
+    <row r="14" ht="61.2" customHeight="1">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="B14" s="41" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>#1462 Eddie (Special Edition 顛倒世界戰鬥 - 有貼紙)
 #1778 Nancy Wheeler (Season 5)
 #1797 Jonathan Byers (Season 5)</t>
         </is>
       </c>
-      <c r="C14" s="41" t="n">
+      <c r="C14" s="40" t="n">
         <v>1800</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="40" t="inlineStr">
+    <row r="15" ht="15.3" customHeight="1">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B15" s="41" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>#804 Dustin (Walmart 限定 夏令營帽子)</t>
         </is>
       </c>
-      <c r="C15" s="41" t="n">
+      <c r="C15" s="40" t="n">
         <v>650</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="40" t="inlineStr">
+    <row r="16" ht="122.4" customHeight="1">
+      <c r="A16" s="39" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B16" s="41" t="inlineStr">
+      <c r="B16" s="40" t="inlineStr">
         <is>
           <t>#514 Nancy (第一季拿槍款)
 #640 Billy (比利經典款)
@@ -3051,50 +3107,51 @@
 #1782 Holly Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="C16" s="41" t="n">
+      <c r="C16" s="40" t="n">
         <v>3600</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="40" t="inlineStr">
+    <row r="17" ht="30.6" customHeight="1">
+      <c r="A17" s="39" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>#1798 Lucas Sinclair (S5 WSQK 特別款)
 #1802 Nancy Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="C17" s="41" t="n">
+      <c r="C17" s="40" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="40" t="inlineStr">
+    <row r="18" ht="45.9" customHeight="1">
+      <c r="A18" s="39" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B18" s="41" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>#428 Demogorgon (魔王開口款)
 #512 Hopper (警長常規款)
-#1810 Holly The Heroic (S5 英雄霍莉)</t>
-        </is>
-      </c>
-      <c r="C18" s="41" t="n">
+#1810 Holly The Heroic (S5 英雄霍莉)
+[備註：與 881/427/550 同買家預訂，預計11月交易]</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="n">
         <v>1200</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="40" t="inlineStr">
+    <row r="19" ht="137.7" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>#476 Mr. Clarke (2017 SDCC 展會限定)
 #513 Jonathan (第一季照相機)
@@ -3105,55 +3162,73 @@
 套組 捉鬼敢死隊 4 人組 (#546, #547, #548, #549)</t>
         </is>
       </c>
-      <c r="C19" s="41" t="n">
+      <c r="C19" s="40" t="n">
         <v>6500</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="40" t="inlineStr">
+    <row r="20" ht="15.3" customHeight="1">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B20" s="41" t="inlineStr">
-        <is>
-          <t>#550 Joyce (磁鐵版)</t>
-        </is>
-      </c>
-      <c r="C20" s="41" t="n">
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>#550 Joyce (磁鐵版)
+[備註：與 881/427/428/512/1810 同買家預訂，預計11月交易]</t>
+        </is>
+      </c>
+      <c r="C20" s="40" t="n">
         <v>400</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="40" t="inlineStr">
+    <row r="21" ht="30.6" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B21" s="41" t="inlineStr">
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>#1780 Eleven (Season 5)
 #1783 Mike Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="C21" s="41" t="n">
+      <c r="C21" s="40" t="n">
         <v>800</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+    <row r="22" ht="30.6" customHeight="1">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B22" s="41" t="inlineStr">
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t>#803 Steve (拿聖代冰淇淋款)
 #922 Robin (拿白板款)</t>
         </is>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C22" s="40" t="n">
         <v>800</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>#427 Barb (第一季經典) (2016購入已絕版)
+#881 Suzie (2019 NYCC 展會限定)
+[備註：與 428/550/512/1810 同買家預訂，預計11月交易]</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="n">
+        <v>1600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>